<commit_message>
Added buses feature changes
</commit_message>
<xml_diff>
--- a/DataSource/TestData.xlsx
+++ b/DataSource/TestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahthati\Desktop\Selenium_June26\Week2\code_7_3\flightbooking\DataSource\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahthati\git\Travelbooking\travelbookingixigo\DataSource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F105D4-61F1-483B-9E29-12975A280F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF4F3E9-E47C-4603-95F8-74A07A2DB10F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3210" yWindow="1070" windowWidth="14380" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TravellerInfo" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="59">
   <si>
     <t>Travel Class</t>
   </si>
@@ -170,9 +170,6 @@
     <t>Departure Date</t>
   </si>
   <si>
-    <t>Bangalore</t>
-  </si>
-  <si>
     <t>Dharma</t>
   </si>
   <si>
@@ -180,6 +177,33 @@
   </si>
   <si>
     <t>Rajiv Gandhi International Airport</t>
+  </si>
+  <si>
+    <t>Boarding point</t>
+  </si>
+  <si>
+    <t>Dropping point</t>
+  </si>
+  <si>
+    <t>Navallur</t>
+  </si>
+  <si>
+    <t>Bengaluru</t>
+  </si>
+  <si>
+    <t>Hayathnagar</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>Rakesh</t>
+  </si>
+  <si>
+    <t>Email</t>
   </si>
 </sst>
 </file>
@@ -586,10 +610,10 @@
         <v>7</v>
       </c>
       <c r="D2" s="3">
-        <v>46217</v>
+        <v>46230</v>
       </c>
       <c r="E2" s="3">
-        <v>46221</v>
+        <v>46233</v>
       </c>
       <c r="F2" t="s">
         <v>14</v>
@@ -639,7 +663,7 @@
         <v>33</v>
       </c>
       <c r="G3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H3" t="s">
         <v>13</v>
@@ -674,10 +698,10 @@
         <v>16</v>
       </c>
       <c r="D4" s="3">
-        <v>46220</v>
+        <v>46231</v>
       </c>
       <c r="E4" s="3">
-        <v>46228</v>
+        <v>46233</v>
       </c>
       <c r="F4" t="s">
         <v>33</v>
@@ -698,10 +722,10 @@
         <v>23</v>
       </c>
       <c r="L4" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4" t="s">
         <v>48</v>
-      </c>
-      <c r="M4" t="s">
-        <v>49</v>
       </c>
       <c r="N4" t="s">
         <v>22</v>
@@ -753,10 +777,10 @@
         <v>42</v>
       </c>
       <c r="C2" s="3">
-        <v>46217</v>
+        <v>46222</v>
       </c>
       <c r="D2" s="3">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -779,7 +803,7 @@
         <v>46227</v>
       </c>
       <c r="D3" s="3">
-        <v>46231</v>
+        <v>46226</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -798,15 +822,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{841C8C8F-3170-4955-BBF0-D2BE67F56D03}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
     <col min="2" max="2" width="10.36328125" customWidth="1"/>
     <col min="3" max="3" width="21.1796875" customWidth="1"/>
+    <col min="5" max="5" width="15.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>44</v>
       </c>
@@ -816,16 +841,60 @@
       <c r="C1" t="s">
         <v>46</v>
       </c>
+      <c r="D1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="C2" s="3">
-        <v>46219</v>
+        <v>46231</v>
+      </c>
+      <c r="D2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2">
+        <v>34</v>
+      </c>
+      <c r="H2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="3">
+        <v>46233</v>
+      </c>
+      <c r="D3" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add gitignore to exclude build artifacts
</commit_message>
<xml_diff>
--- a/DataSource/TestData.xlsx
+++ b/DataSource/TestData.xlsx
@@ -3,24 +3,23 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahthati\git\Travelbooking\travelbookingixigo\DataSource\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF4F3E9-E47C-4603-95F8-74A07A2DB10F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{E4191103-57E9-4300-BCA8-676E077EDBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3210" yWindow="1070" windowWidth="14380" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TravellerInfo" sheetId="1" r:id="rId1"/>
     <sheet name="HotelBooking" sheetId="2" r:id="rId2"/>
     <sheet name="BusBooking" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:E8"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
     </ext>
   </extLst>
 </workbook>

</xml_diff>

<commit_message>
Updatereport: updated runner for report
</commit_message>
<xml_diff>
--- a/DataSource/TestData.xlsx
+++ b/DataSource/TestData.xlsx
@@ -3,9 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{E4191103-57E9-4300-BCA8-676E077EDBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahthati\git\Travelbooking\travelbookingixigo\DataSource\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B42981A0-FA4E-4C4F-B1C1-0F728C4E58D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TravellerInfo" sheetId="1" r:id="rId1"/>
@@ -13,7 +18,6 @@
     <sheet name="BusBooking" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:E8"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -776,10 +780,10 @@
         <v>42</v>
       </c>
       <c r="C2" s="3">
-        <v>46222</v>
+        <v>46226</v>
       </c>
       <c r="D2" s="3">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -799,10 +803,10 @@
         <v>43</v>
       </c>
       <c r="C3" s="3">
+        <v>46226</v>
+      </c>
+      <c r="D3" s="3">
         <v>46227</v>
-      </c>
-      <c r="D3" s="3">
-        <v>46226</v>
       </c>
       <c r="E3">
         <v>1</v>

</xml_diff>

<commit_message>
flightsEx: updated runner for flights execution
</commit_message>
<xml_diff>
--- a/DataSource/TestData.xlsx
+++ b/DataSource/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahthati\git\Travelbooking\travelbookingixigo\DataSource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B42981A0-FA4E-4C4F-B1C1-0F728C4E58D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80DEA8CD-AD71-437C-A493-0C10087FEE78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TravellerInfo" sheetId="1" r:id="rId1"/>

</xml_diff>